<commit_message>
cleaned pre trend data
</commit_message>
<xml_diff>
--- a/Solar 2010.xlsx
+++ b/Solar 2010.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfc87df69086cb6c/Desktop/Green Bonds Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C84BD7E8-3404-409D-B649-DDB42873A128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{C84BD7E8-3404-409D-B649-DDB42873A128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75EEB121-F0B0-48A3-BAED-F7B7E2D81AD6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>CO</t>
   </si>
@@ -49,13 +49,10 @@
     <t>TX</t>
   </si>
   <si>
-    <t>2010</t>
-  </si>
-  <si>
     <t>State</t>
   </si>
   <si>
-    <t>Year</t>
+    <t>Capacity</t>
   </si>
 </sst>
 </file>
@@ -84,14 +81,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -131,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -142,10 +132,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -163,6 +150,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -482,91 +473,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
-        <v>11</v>
+      <c r="A1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="5">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>22.6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5">
-        <v>22.6</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>8.25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5">
-        <v>8.25</v>
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>17.5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5">
-        <v>17.5</v>
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="5">
-        <v>5.0999999999999996</v>
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>30.64</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="5">
-        <v>30.64</v>
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="5">
-        <v>48</v>
+        <v>7</v>
+      </c>
+      <c r="B9" s="4">
+        <v>10.08</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="5">
-        <v>10.08</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B10" s="4">
         <v>13.9</v>
       </c>
     </row>

</xml_diff>